<commit_message>
Update Excel file links and row counts in Vilande kursplaner for IKS, ISLL, and IIT
</commit_message>
<xml_diff>
--- a/vault-dalarna-university/03 IKS/Analys/Vilande kursplaner.xlsx
+++ b/vault-dalarna-university/03 IKS/Analys/Vilande kursplaner.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Vilande kursplaner" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Vilande kursplaner'!$A$1:$H$14</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Vilande kursplaner'!$A$1:$H$8</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -432,7 +432,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H14"/>
+  <dimension ref="A1:H8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -490,32 +490,32 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>BY1047</t>
+          <t>AHI29Q</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>BYA</t>
+          <t>HIA</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>IIT</t>
+          <t>IKS</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>2013-03-14</t>
+          <t>2023-10-05</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>Byggteknik</t>
+          <t>Historia</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>Bärkraftigt byggande och boende</t>
+          <t>Historievetenskaplig litteraturkurs</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
@@ -525,39 +525,39 @@
       </c>
       <c r="H2" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=BY1047</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=AHI29Q</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>GIK289</t>
+          <t>AHI29R</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>IKA</t>
+          <t>HIA</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>IIT</t>
+          <t>IKS</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>2019-02-21</t>
+          <t>2023-10-05</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Informatik</t>
+          <t>Historia</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>Objektorienterad programmering och problemlösning</t>
+          <t>Historievetenskapens teori och metod</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
@@ -567,39 +567,39 @@
       </c>
       <c r="H3" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIK289</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=AHI29R</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>GRY2BR</t>
+          <t>GFI37Z</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>RYA</t>
+          <t>FIA</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>ISLL</t>
+          <t>IKS</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>2019-10-09</t>
+          <t>2023-12-07</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>Ryska</t>
+          <t>Filosofi</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>Ryska V: Samtida rysk litteratur och kultur</t>
+          <t>Gud och bevisen: filosofiska argument för och mot Guds existens</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
@@ -609,39 +609,39 @@
       </c>
       <c r="H4" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GRY2BR</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GFI37Z</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>GKI2W3</t>
+          <t>GPG3CN</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>KIA</t>
+          <t>PGA</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>ISLL</t>
+          <t>IKS</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>2022-04-28</t>
+          <t>2024-09-05</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Kinesiska</t>
+          <t>Pedagogiskt arbete</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>Kinesiska I med didaktisk inriktning</t>
+          <t>Undervisning och lärande genom rollspel - inriktning pedagogiskt arbete</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
@@ -651,14 +651,14 @@
       </c>
       <c r="H5" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GKI2W3</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GPG3CN</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>AHI29Q</t>
+          <t>GHI3CP</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -673,7 +673,7 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>2023-10-05</t>
+          <t>2024-09-27</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
@@ -683,7 +683,7 @@
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>Historievetenskaplig litteraturkurs</t>
+          <t>Undervisning och lärande genom rollspel – inriktning historiedidaktik</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
@@ -693,19 +693,19 @@
       </c>
       <c r="H6" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=AHI29Q</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GHI3CP</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>AHI29R</t>
+          <t>GRK3CQ</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>HIA</t>
+          <t>RKA</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -715,17 +715,17 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>2023-10-05</t>
+          <t>2024-09-27</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>Historia</t>
+          <t>Religionsvetenskap</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>Historievetenskapens teori och metod</t>
+          <t>Undervisning och lärande genom rollspel – inriktning religionsdidaktik</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
@@ -735,19 +735,19 @@
       </c>
       <c r="H7" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=AHI29R</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GRK3CQ</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>GFI37Z</t>
+          <t>APG2CC</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>FIA</t>
+          <t>PGA</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -757,17 +757,17 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>2023-12-07</t>
+          <t>2026-02-23</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>Filosofi</t>
+          <t>Pedagogiskt arbete</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>Gud och bevisen: filosofiska argument för och mot Guds existens</t>
+          <t>Mentorsutbildning för en kvalitativ introduktionsperiod</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
@@ -776,265 +776,13 @@
         </is>
       </c>
       <c r="H8" s="2" t="inlineStr">
-        <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GFI37Z</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="2" t="inlineStr">
-        <is>
-          <t>GIH3AQ</t>
-        </is>
-      </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>IDA</t>
-        </is>
-      </c>
-      <c r="C9" t="inlineStr">
-        <is>
-          <t>IHV</t>
-        </is>
-      </c>
-      <c r="D9" t="inlineStr">
-        <is>
-          <t>2024-02-27</t>
-        </is>
-      </c>
-      <c r="E9" t="inlineStr">
-        <is>
-          <t>Idrotts- och hälsovetenskap</t>
-        </is>
-      </c>
-      <c r="F9" t="inlineStr">
-        <is>
-          <t>Styrketräningens teori och praktiska tillämpning</t>
-        </is>
-      </c>
-      <c r="G9" t="inlineStr">
-        <is>
-          <t>Ingen aktiv kursomgång hittad på kurssidan</t>
-        </is>
-      </c>
-      <c r="H9" s="2" t="inlineStr">
-        <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIH3AQ</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="2" t="inlineStr">
-        <is>
-          <t>GKI3C9</t>
-        </is>
-      </c>
-      <c r="B10" t="inlineStr">
-        <is>
-          <t>KIA</t>
-        </is>
-      </c>
-      <c r="C10" t="inlineStr">
-        <is>
-          <t>ISLL</t>
-        </is>
-      </c>
-      <c r="D10" t="inlineStr">
-        <is>
-          <t>2024-06-19</t>
-        </is>
-      </c>
-      <c r="E10" t="inlineStr">
-        <is>
-          <t>Kinesiska</t>
-        </is>
-      </c>
-      <c r="F10" t="inlineStr">
-        <is>
-          <t>Kinesiska för affärslivet II</t>
-        </is>
-      </c>
-      <c r="G10" t="inlineStr">
-        <is>
-          <t>Ingen aktiv kursomgång hittad på kurssidan</t>
-        </is>
-      </c>
-      <c r="H10" s="2" t="inlineStr">
-        <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GKI3C9</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="2" t="inlineStr">
-        <is>
-          <t>GPG3CN</t>
-        </is>
-      </c>
-      <c r="B11" t="inlineStr">
-        <is>
-          <t>PGA</t>
-        </is>
-      </c>
-      <c r="C11" t="inlineStr">
-        <is>
-          <t>IKS</t>
-        </is>
-      </c>
-      <c r="D11" t="inlineStr">
-        <is>
-          <t>2024-09-05</t>
-        </is>
-      </c>
-      <c r="E11" t="inlineStr">
-        <is>
-          <t>Pedagogiskt arbete</t>
-        </is>
-      </c>
-      <c r="F11" t="inlineStr">
-        <is>
-          <t>Undervisning och lärande genom rollspel - inriktning pedagogiskt arbete</t>
-        </is>
-      </c>
-      <c r="G11" t="inlineStr">
-        <is>
-          <t>Ingen aktiv kursomgång hittad på kurssidan</t>
-        </is>
-      </c>
-      <c r="H11" s="2" t="inlineStr">
-        <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GPG3CN</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="2" t="inlineStr">
-        <is>
-          <t>GHI3CP</t>
-        </is>
-      </c>
-      <c r="B12" t="inlineStr">
-        <is>
-          <t>HIA</t>
-        </is>
-      </c>
-      <c r="C12" t="inlineStr">
-        <is>
-          <t>IKS</t>
-        </is>
-      </c>
-      <c r="D12" t="inlineStr">
-        <is>
-          <t>2024-09-27</t>
-        </is>
-      </c>
-      <c r="E12" t="inlineStr">
-        <is>
-          <t>Historia</t>
-        </is>
-      </c>
-      <c r="F12" t="inlineStr">
-        <is>
-          <t>Undervisning och lärande genom rollspel – inriktning historiedidaktik</t>
-        </is>
-      </c>
-      <c r="G12" t="inlineStr">
-        <is>
-          <t>Ingen aktiv kursomgång hittad på kurssidan</t>
-        </is>
-      </c>
-      <c r="H12" s="2" t="inlineStr">
-        <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GHI3CP</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="2" t="inlineStr">
-        <is>
-          <t>GRK3CQ</t>
-        </is>
-      </c>
-      <c r="B13" t="inlineStr">
-        <is>
-          <t>RKA</t>
-        </is>
-      </c>
-      <c r="C13" t="inlineStr">
-        <is>
-          <t>IKS</t>
-        </is>
-      </c>
-      <c r="D13" t="inlineStr">
-        <is>
-          <t>2024-09-27</t>
-        </is>
-      </c>
-      <c r="E13" t="inlineStr">
-        <is>
-          <t>Religionsvetenskap</t>
-        </is>
-      </c>
-      <c r="F13" t="inlineStr">
-        <is>
-          <t>Undervisning och lärande genom rollspel – inriktning religionsdidaktik</t>
-        </is>
-      </c>
-      <c r="G13" t="inlineStr">
-        <is>
-          <t>Ingen aktiv kursomgång hittad på kurssidan</t>
-        </is>
-      </c>
-      <c r="H13" s="2" t="inlineStr">
-        <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GRK3CQ</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="2" t="inlineStr">
-        <is>
-          <t>APG2CC</t>
-        </is>
-      </c>
-      <c r="B14" t="inlineStr">
-        <is>
-          <t>PGA</t>
-        </is>
-      </c>
-      <c r="C14" t="inlineStr">
-        <is>
-          <t>IKS</t>
-        </is>
-      </c>
-      <c r="D14" t="inlineStr">
-        <is>
-          <t>2026-02-23</t>
-        </is>
-      </c>
-      <c r="E14" t="inlineStr">
-        <is>
-          <t>Pedagogiskt arbete</t>
-        </is>
-      </c>
-      <c r="F14" t="inlineStr">
-        <is>
-          <t>Mentorsutbildning för en kvalitativ introduktionsperiod</t>
-        </is>
-      </c>
-      <c r="G14" t="inlineStr">
-        <is>
-          <t>Ingen aktiv kursomgång hittad på kurssidan</t>
-        </is>
-      </c>
-      <c r="H14" s="2" t="inlineStr">
         <is>
           <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=APG2CC</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:H14"/>
+  <autoFilter ref="A1:H8"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H2" r:id="rId2"/>
@@ -1050,18 +798,6 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H7" r:id="rId12"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A8" r:id="rId13"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H8" r:id="rId14"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A9" r:id="rId15"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H9" r:id="rId16"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A10" r:id="rId17"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H10" r:id="rId18"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A11" r:id="rId19"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H11" r:id="rId20"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A12" r:id="rId21"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H12" r:id="rId22"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A13" r:id="rId23"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H13" r:id="rId24"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A14" r:id="rId25"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H14" r:id="rId26"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>